<commit_message>
Add Oct 28 analyses and update reverse DCF workbook
- Price per Gb by machine (Illumina and competitors)
- Competitor H2 2026 sequencing launches with price per Gb
- Writeup edit list for the UIC pitch
- Latest saved version of the reverse DCF workbook

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Working Notes/Outputs/datasets/2026-10-13_ILMN_reverse_DCF.xlsx
+++ b/Working Notes/Outputs/datasets/2026-10-13_ILMN_reverse_DCF.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ec57dbfba1bbe215/Documents/ILMN Claude Code Local Folder/Working Notes/Outputs/datasets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="252" documentId="11_EBC793924E84E83F2F9EA82992EA9A596B41CE07" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AFA02F0F-7062-4A2E-B090-80D7CC3AAA4D}"/>
+  <xr:revisionPtr revIDLastSave="265" documentId="11_EBC793924E84E83F2F9EA82992EA9A596B41CE07" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0EDE062E-31B0-42BF-B1B2-BBE119AA72A1}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,7 +43,7 @@
     <definedName name="IQ_YTD">3000</definedName>
     <definedName name="IQ_YTDMONTH" hidden="1">130000</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="9.9999999999994451E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -681,7 +681,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -702,17 +702,6 @@
       <left style="dashed">
         <color rgb="FFC00000"/>
       </left>
-      <right/>
-      <top style="dashed">
-        <color rgb="FFC00000"/>
-      </top>
-      <bottom style="dashed">
-        <color rgb="FFC00000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="dashed">
         <color rgb="FFC00000"/>
@@ -748,15 +737,6 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top style="dashed">
-        <color rgb="FFC00000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="dashed">
         <color rgb="FFC00000"/>
       </right>
@@ -779,15 +759,6 @@
     </border>
     <border>
       <left/>
-      <right/>
-      <top/>
-      <bottom style="dashed">
-        <color rgb="FFC00000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="dashed">
         <color rgb="FFC00000"/>
       </right>
@@ -801,7 +772,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -854,18 +825,15 @@
     <xf numFmtId="164" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="10" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="10" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="10" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="12" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="10" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="13" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="15" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="15" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="15" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="10" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1178,6 +1146,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="700" row="7">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{0641BBE8-54B3-45B8-BA44-735830C6ACD8}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;a55566d8-bc41-4963-a04d-e781e08ea586&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L88"/>
@@ -1268,7 +1258,7 @@
       <c r="K5" s="34" t="s">
         <v>10</v>
       </c>
-      <c r="L5" s="56">
+      <c r="L5" s="53">
         <f>(B24*I61+B32)/I13</f>
         <v>20.577370656858715</v>
       </c>
@@ -1282,27 +1272,27 @@
         <f t="shared" ref="C6:I6" si="0">C5/B5-1</f>
         <v>2.5392428439519055E-3</v>
       </c>
-      <c r="D6" s="53">
+      <c r="D6" s="51">
         <f t="shared" si="0"/>
         <v>6.3780796684319574E-2</v>
       </c>
-      <c r="E6" s="54">
+      <c r="E6" s="52">
         <f t="shared" si="0"/>
         <v>0.13946729091412813</v>
       </c>
-      <c r="F6" s="54">
+      <c r="F6" s="36">
         <f t="shared" si="0"/>
         <v>0.13946729091412813</v>
       </c>
-      <c r="G6" s="54">
+      <c r="G6" s="36">
         <f t="shared" si="0"/>
         <v>0.13946729091412813</v>
       </c>
-      <c r="H6" s="54">
+      <c r="H6" s="36">
         <f t="shared" si="0"/>
         <v>0.13946729091412813</v>
       </c>
-      <c r="I6" s="55">
+      <c r="I6" s="36">
         <f t="shared" si="0"/>
         <v>0.13946729091412813</v>
       </c>
@@ -1316,33 +1306,33 @@
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A7" s="65" t="s">
+      <c r="A7" s="62" t="s">
         <v>99</v>
       </c>
-      <c r="B7" s="66"/>
-      <c r="C7" s="66"/>
-      <c r="D7" s="67">
-        <f>ROUND((D6-D84)*10000,0)</f>
+      <c r="B7" s="63"/>
+      <c r="C7" s="63"/>
+      <c r="D7" s="64">
+        <f t="shared" ref="D7:I7" si="1">ROUND((D6-D84)*10000,0)</f>
         <v>-12</v>
       </c>
-      <c r="E7" s="67">
-        <f>ROUND((E6-E84)*10000,0)</f>
+      <c r="E7" s="64">
+        <f t="shared" si="1"/>
         <v>761</v>
       </c>
-      <c r="F7" s="67">
-        <f>ROUND((F6-F84)*10000,0)</f>
+      <c r="F7" s="64">
+        <f t="shared" si="1"/>
         <v>693</v>
       </c>
-      <c r="G7" s="67">
-        <f>ROUND((G6-G84)*10000,0)</f>
+      <c r="G7" s="64">
+        <f t="shared" si="1"/>
         <v>659</v>
       </c>
-      <c r="H7" s="67">
-        <f>ROUND((H6-H84)*10000,0)</f>
+      <c r="H7" s="64">
+        <f t="shared" si="1"/>
         <v>619</v>
       </c>
-      <c r="I7" s="67">
-        <f>ROUND((I6-I84)*10000,0)</f>
+      <c r="I7" s="64">
+        <f t="shared" si="1"/>
         <v>383</v>
       </c>
       <c r="J7" s="30"/>
@@ -1359,35 +1349,35 @@
         <v>13</v>
       </c>
       <c r="B8" s="39">
-        <f t="shared" ref="B8:I8" si="1">-(B5-B9)</f>
+        <f t="shared" ref="B8:I8" si="2">-(B5-B9)</f>
         <v>-1360</v>
       </c>
       <c r="C8" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1379</v>
       </c>
       <c r="D8" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1455.2999999999997</v>
       </c>
       <c r="E8" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1626.6807151631915</v>
       </c>
       <c r="F8" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-1829.5552998227304</v>
       </c>
       <c r="G8" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-2050.5427092458285</v>
       </c>
       <c r="H8" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-2313.1610823499796</v>
       </c>
       <c r="I8" s="39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>-2591.3981361965343</v>
       </c>
       <c r="J8" s="30"/>
@@ -1410,27 +1400,27 @@
         <v>2964</v>
       </c>
       <c r="D9" s="33">
-        <f t="shared" ref="D9:I9" si="2">D5*D39</f>
+        <f t="shared" ref="D9:I9" si="3">D5*D39</f>
         <v>3164.7000000000003</v>
       </c>
       <c r="E9" s="33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3637.6581688600804</v>
       </c>
       <c r="F9" s="33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4168.9866668091718</v>
       </c>
       <c r="G9" s="33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4784.5996549069314</v>
       </c>
       <c r="H9" s="33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5475.2600703435546</v>
       </c>
       <c r="I9" s="33">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6283.2530151614574</v>
       </c>
       <c r="J9" s="30"/>
@@ -1447,35 +1437,35 @@
         <v>17</v>
       </c>
       <c r="B10" s="36">
-        <f t="shared" ref="B10:I10" si="3">B9/B5</f>
+        <f t="shared" ref="B10:I10" si="4">B9/B5</f>
         <v>0.68605724838411819</v>
       </c>
       <c r="C10" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.68247755008058941</v>
       </c>
       <c r="D10" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.68500000000000005</v>
       </c>
       <c r="E10" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.69099999999999995</v>
       </c>
       <c r="F10" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.69499999999999995</v>
       </c>
       <c r="G10" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.7</v>
       </c>
       <c r="H10" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.70299999999999996</v>
       </c>
       <c r="I10" s="36">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.70799999999999996</v>
       </c>
       <c r="J10" s="30"/>
@@ -1488,33 +1478,33 @@
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A11" s="62" t="s">
+      <c r="A11" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="63"/>
-      <c r="C11" s="63"/>
-      <c r="D11" s="64">
-        <f>ROUND((D10-D85)*10000,0)</f>
+      <c r="B11" s="60"/>
+      <c r="C11" s="60"/>
+      <c r="D11" s="61">
+        <f t="shared" ref="D11:I11" si="5">ROUND((D10-D85)*10000,0)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="64">
-        <f>ROUND((E10-E85)*10000,0)</f>
+      <c r="E11" s="61">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="F11" s="64">
-        <f>ROUND((F10-F85)*10000,0)</f>
+      <c r="F11" s="61">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="G11" s="64">
-        <f>ROUND((G10-G85)*10000,0)</f>
+      <c r="G11" s="61">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="H11" s="64">
-        <f>ROUND((H10-H85)*10000,0)</f>
+      <c r="H11" s="61">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I11" s="64">
-        <f>ROUND((I10-I85)*10000,0)</f>
+      <c r="I11" s="61">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J11" s="30"/>
@@ -1531,35 +1521,35 @@
         <v>19</v>
       </c>
       <c r="B12" s="39">
-        <f t="shared" ref="B12:I12" si="4">-(B9-B13)</f>
+        <f t="shared" ref="B12:I12" si="6">-(B9-B13)</f>
         <v>-1825</v>
       </c>
       <c r="C12" s="39">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>-1756</v>
       </c>
       <c r="D12" s="39">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>-1867.1043243243248</v>
       </c>
       <c r="E12" s="39">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>-2042.7283320982515</v>
       </c>
       <c r="F12" s="39">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>-2319.1607857824611</v>
       </c>
       <c r="G12" s="39">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>-2617.9200134560301</v>
       </c>
       <c r="H12" s="39">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>-2920.4839465050218</v>
       </c>
       <c r="I12" s="39">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>-3409.3169099111292</v>
       </c>
       <c r="J12" s="30"/>
@@ -1582,34 +1572,34 @@
         <v>1208</v>
       </c>
       <c r="D13" s="39">
-        <f t="shared" ref="D13:I13" si="5">D5*(D40+D41)</f>
+        <f t="shared" ref="D13:I13" si="7">D5*(D40+D41)</f>
         <v>1297.5956756756755</v>
       </c>
       <c r="E13" s="39">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1594.9298367618289</v>
       </c>
       <c r="F13" s="39">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>1849.8258810267107</v>
       </c>
       <c r="G13" s="39">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>2166.6796414509013</v>
       </c>
       <c r="H13" s="39">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>2554.7761238385328</v>
       </c>
       <c r="I13" s="39">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>2873.9361052503282</v>
       </c>
       <c r="J13" s="30"/>
       <c r="K13" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="L13" s="47">
+      <c r="L13" s="46">
         <f>L11/L12</f>
         <v>271.7600000000001</v>
       </c>
@@ -1619,74 +1609,74 @@
         <v>23</v>
       </c>
       <c r="B14" s="36">
-        <f t="shared" ref="B14:I14" si="6">B13/B5</f>
+        <f t="shared" ref="B14:I14" si="8">B13/B5</f>
         <v>0.26477377654662976</v>
       </c>
       <c r="C14" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.27814874510706883</v>
       </c>
       <c r="D14" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.28086486486486484</v>
       </c>
       <c r="E14" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.3029686864579097</v>
       </c>
       <c r="F14" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.30837925137754135</v>
       </c>
       <c r="G14" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.31699115044247783</v>
       </c>
       <c r="H14" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.32802233902759526</v>
       </c>
       <c r="I14" s="36">
-        <f t="shared" si="6"/>
+        <f t="shared" si="8"/>
         <v>0.32383651551312648</v>
       </c>
       <c r="J14" s="30"/>
-      <c r="K14" s="51" t="s">
+      <c r="K14" s="49" t="s">
         <v>28</v>
       </c>
-      <c r="L14" s="52">
+      <c r="L14" s="50">
         <f>L13/B21-1</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.45">
-      <c r="A15" s="62" t="s">
+      <c r="A15" s="59" t="s">
         <v>99</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="64">
-        <f>ROUND((D14-D87)*10000,0)</f>
+      <c r="B15" s="60"/>
+      <c r="C15" s="60"/>
+      <c r="D15" s="61">
+        <f t="shared" ref="D15:I15" si="9">ROUND((D14-D87)*10000,0)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="64">
-        <f>ROUND((E14-E87)*10000,0)</f>
+      <c r="E15" s="61">
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="F15" s="64">
-        <f>ROUND((F14-F87)*10000,0)</f>
+      <c r="F15" s="61">
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="G15" s="64">
-        <f>ROUND((G14-G87)*10000,0)</f>
+      <c r="G15" s="61">
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="H15" s="64">
-        <f>ROUND((H14-H87)*10000,0)</f>
+      <c r="H15" s="61">
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="I15" s="64">
-        <f>ROUND((I14-I87)*10000,0)</f>
+      <c r="I15" s="61">
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="J15" s="30"/>
@@ -1696,35 +1686,35 @@
         <v>25</v>
       </c>
       <c r="B16" s="43">
-        <f t="shared" ref="B16:I16" si="7">(1+B43)/(1+$B$34)-1</f>
+        <f t="shared" ref="B16:I16" si="10">(1+B43)/(1+$B$34)-1</f>
         <v>-0.1764874551971326</v>
       </c>
       <c r="C16" s="43">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>-0.18133704735376044</v>
       </c>
       <c r="D16" s="44">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>-0.1489753626525443</v>
       </c>
       <c r="E16" s="45">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>-8.8426167268697342E-2</v>
       </c>
-      <c r="F16" s="45">
-        <f t="shared" si="7"/>
+      <c r="F16" s="43">
+        <f t="shared" si="10"/>
         <v>-8.8426167268697453E-2</v>
       </c>
-      <c r="G16" s="45">
-        <f t="shared" si="7"/>
+      <c r="G16" s="43">
+        <f t="shared" si="10"/>
         <v>-8.8426167268697675E-2</v>
       </c>
-      <c r="H16" s="45">
-        <f t="shared" si="7"/>
+      <c r="H16" s="43">
+        <f t="shared" si="10"/>
         <v>-8.8426167268697342E-2</v>
       </c>
-      <c r="I16" s="46">
-        <f t="shared" si="7"/>
+      <c r="I16" s="43">
+        <f t="shared" si="10"/>
         <v>-8.8426167268697675E-2</v>
       </c>
       <c r="J16" s="30"/>
@@ -1734,35 +1724,35 @@
         <v>27</v>
       </c>
       <c r="B17" s="43">
-        <f t="shared" ref="B17:I17" si="8">(1+B43)/(1+$B$35)-1</f>
+        <f t="shared" ref="B17:I17" si="11">(1+B43)/(1+$B$35)-1</f>
         <v>-0.20816101461262759</v>
       </c>
       <c r="C17" s="43">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>-0.21282408399400043</v>
       </c>
-      <c r="D17" s="48">
-        <f t="shared" si="8"/>
+      <c r="D17" s="47">
+        <f t="shared" si="11"/>
         <v>-0.18170707947360032</v>
       </c>
-      <c r="E17" s="49">
-        <f t="shared" si="8"/>
+      <c r="E17" s="48">
+        <f t="shared" si="11"/>
         <v>-0.12348669929682443</v>
       </c>
-      <c r="F17" s="49">
-        <f t="shared" si="8"/>
+      <c r="F17" s="43">
+        <f t="shared" si="11"/>
         <v>-0.12348669929682454</v>
       </c>
-      <c r="G17" s="49">
-        <f t="shared" si="8"/>
+      <c r="G17" s="43">
+        <f t="shared" si="11"/>
         <v>-0.12348669929682476</v>
       </c>
-      <c r="H17" s="49">
-        <f t="shared" si="8"/>
+      <c r="H17" s="43">
+        <f t="shared" si="11"/>
         <v>-0.12348669929682443</v>
       </c>
-      <c r="I17" s="50">
-        <f t="shared" si="8"/>
+      <c r="I17" s="43">
+        <f t="shared" si="11"/>
         <v>-0.12348669929682476</v>
       </c>
       <c r="J17" s="30"/>
@@ -2004,28 +1994,28 @@
         <f>C9/C5</f>
         <v>0.68247755008058941</v>
       </c>
-      <c r="D39" s="58">
-        <f t="shared" ref="D39:I39" si="9">D85</f>
+      <c r="D39" s="55">
+        <f t="shared" ref="D39:I39" si="12">D85</f>
         <v>0.68500000000000005</v>
       </c>
-      <c r="E39" s="58">
-        <f t="shared" si="9"/>
+      <c r="E39" s="55">
+        <f t="shared" si="12"/>
         <v>0.69099999999999995</v>
       </c>
-      <c r="F39" s="58">
-        <f t="shared" si="9"/>
+      <c r="F39" s="55">
+        <f t="shared" si="12"/>
         <v>0.69499999999999995</v>
       </c>
-      <c r="G39" s="58">
-        <f t="shared" si="9"/>
+      <c r="G39" s="55">
+        <f t="shared" si="12"/>
         <v>0.7</v>
       </c>
-      <c r="H39" s="58">
-        <f t="shared" si="9"/>
+      <c r="H39" s="55">
+        <f t="shared" si="12"/>
         <v>0.70299999999999996</v>
       </c>
-      <c r="I39" s="58">
-        <f t="shared" si="9"/>
+      <c r="I39" s="55">
+        <f t="shared" si="12"/>
         <v>0.70799999999999996</v>
       </c>
       <c r="J39" s="13" t="s">
@@ -2043,28 +2033,28 @@
         <f>1004/C5</f>
         <v>0.2311766060326963</v>
       </c>
-      <c r="D40" s="58">
-        <f t="shared" ref="D40:I40" si="10">D87-D41</f>
+      <c r="D40" s="55">
+        <f t="shared" ref="D40:I40" si="13">D87-D41</f>
         <v>0.23486486486486485</v>
       </c>
-      <c r="E40" s="58">
-        <f t="shared" si="10"/>
+      <c r="E40" s="55">
+        <f t="shared" si="13"/>
         <v>0.25796868645790971</v>
       </c>
-      <c r="F40" s="58">
-        <f t="shared" si="10"/>
+      <c r="F40" s="55">
+        <f t="shared" si="13"/>
         <v>0.26437925137754137</v>
       </c>
-      <c r="G40" s="58">
-        <f t="shared" si="10"/>
+      <c r="G40" s="55">
+        <f t="shared" si="13"/>
         <v>0.2739911504424779</v>
       </c>
-      <c r="H40" s="58">
-        <f t="shared" si="10"/>
+      <c r="H40" s="55">
+        <f t="shared" si="13"/>
         <v>0.28602233902759527</v>
       </c>
-      <c r="I40" s="58">
-        <f t="shared" si="10"/>
+      <c r="I40" s="55">
+        <f t="shared" si="13"/>
         <v>0.2828365155131265</v>
       </c>
       <c r="J40" s="13" t="s">
@@ -2116,27 +2106,27 @@
         <v>2939</v>
       </c>
       <c r="D42" s="8">
-        <f t="shared" ref="D42:I42" si="11">D5*$C$42/$C$5</f>
+        <f t="shared" ref="D42:I42" si="14">D5*$C$42/$C$5</f>
         <v>3126.4517614552151</v>
       </c>
       <c r="E42" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>3562.4895187990783</v>
       </c>
       <c r="F42" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>4059.3402808959613</v>
       </c>
       <c r="G42" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>4625.4854727711163</v>
       </c>
       <c r="H42" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>5270.5894008211599</v>
       </c>
       <c r="I42" s="8">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>6005.6642260744038</v>
       </c>
       <c r="J42" s="13" t="s">
@@ -2152,31 +2142,31 @@
         <v>2.9390681003584218E-2</v>
       </c>
       <c r="C43" s="19">
-        <f t="shared" ref="C43:I43" si="12">C42/B42-1</f>
+        <f t="shared" ref="C43:I43" si="15">C42/B42-1</f>
         <v>2.3328690807799424E-2</v>
       </c>
       <c r="D43" s="19">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>6.3780796684319574E-2</v>
       </c>
       <c r="E43" s="19">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.13946729091412835</v>
       </c>
       <c r="F43" s="19">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.13946729091412813</v>
       </c>
       <c r="G43" s="19">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.13946729091412791</v>
       </c>
       <c r="H43" s="19">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.13946729091412835</v>
       </c>
       <c r="I43" s="19">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>0.13946729091412791</v>
       </c>
     </row>
@@ -2231,27 +2221,27 @@
         <v>21</v>
       </c>
       <c r="D47" s="8">
-        <f t="shared" ref="D47:I47" si="13">D13</f>
+        <f t="shared" ref="D47:I47" si="16">D13</f>
         <v>1297.5956756756755</v>
       </c>
       <c r="E47" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1594.9298367618289</v>
       </c>
       <c r="F47" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1849.8258810267107</v>
       </c>
       <c r="G47" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>2166.6796414509013</v>
       </c>
       <c r="H47" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>2554.7761238385328</v>
       </c>
       <c r="I47" s="8">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>2873.9361052503282</v>
       </c>
     </row>
@@ -2260,27 +2250,27 @@
         <v>74</v>
       </c>
       <c r="D48" s="8">
-        <f t="shared" ref="D48:I48" si="14">-D5*D41</f>
+        <f t="shared" ref="D48:I48" si="17">-D5*D41</f>
         <v>-212.52</v>
       </c>
       <c r="E48" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>-236.89524978104723</v>
       </c>
       <c r="F48" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>-263.93584653180369</v>
       </c>
       <c r="G48" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>-293.91112165856867</v>
       </c>
       <c r="H48" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>-327.11368841312844</v>
       </c>
       <c r="I48" s="8">
-        <f t="shared" si="14"/>
+        <f t="shared" si="17"/>
         <v>-363.8606972056777</v>
       </c>
     </row>
@@ -2289,27 +2279,27 @@
         <v>75</v>
       </c>
       <c r="D49" s="8">
-        <f t="shared" ref="D49:I49" si="15">D47+D48</f>
+        <f t="shared" ref="D49:I49" si="18">D47+D48</f>
         <v>1085.0756756756755</v>
       </c>
       <c r="E49" s="8">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>1358.0345869807818</v>
       </c>
       <c r="F49" s="8">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>1585.890034494907</v>
       </c>
       <c r="G49" s="8">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>1872.7685197923327</v>
       </c>
       <c r="H49" s="8">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>2227.6624354254045</v>
       </c>
       <c r="I49" s="8">
-        <f t="shared" si="15"/>
+        <f t="shared" si="18"/>
         <v>2510.0754080446504</v>
       </c>
     </row>
@@ -2318,27 +2308,27 @@
         <v>76</v>
       </c>
       <c r="D50" s="8">
-        <f t="shared" ref="D50:I50" si="16">-D49*$B$27</f>
+        <f t="shared" ref="D50:I50" si="19">-D49*$B$27</f>
         <v>-222.44051351351345</v>
       </c>
       <c r="E50" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>-278.39709033106027</v>
       </c>
       <c r="F50" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>-325.10745707145594</v>
       </c>
       <c r="G50" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>-383.91754655742818</v>
       </c>
       <c r="H50" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>-456.67079926220788</v>
       </c>
       <c r="I50" s="8">
-        <f t="shared" si="16"/>
+        <f t="shared" si="19"/>
         <v>-514.56545864915336</v>
       </c>
     </row>
@@ -2347,27 +2337,27 @@
         <v>77</v>
       </c>
       <c r="D51" s="8">
-        <f t="shared" ref="D51:I51" si="17">-D48</f>
+        <f t="shared" ref="D51:I51" si="20">-D48</f>
         <v>212.52</v>
       </c>
       <c r="E51" s="8">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>236.89524978104723</v>
       </c>
       <c r="F51" s="8">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>263.93584653180369</v>
       </c>
       <c r="G51" s="8">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>293.91112165856867</v>
       </c>
       <c r="H51" s="8">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>327.11368841312844</v>
       </c>
       <c r="I51" s="8">
-        <f t="shared" si="17"/>
+        <f t="shared" si="20"/>
         <v>363.8606972056777</v>
       </c>
     </row>
@@ -2376,27 +2366,27 @@
         <v>78</v>
       </c>
       <c r="D52" s="8">
-        <f t="shared" ref="D52:I52" si="18">-D5*$B$28</f>
+        <f t="shared" ref="D52:I52" si="21">-D5*$B$28</f>
         <v>-226.38</v>
       </c>
       <c r="E52" s="8">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>-257.95260531714035</v>
       </c>
       <c r="F52" s="8">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>-293.92855636496324</v>
       </c>
       <c r="G52" s="8">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>-334.92197584348526</v>
       </c>
       <c r="H52" s="8">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>-381.63263648198318</v>
       </c>
       <c r="I52" s="8">
-        <f t="shared" si="18"/>
+        <f t="shared" si="21"/>
         <v>-434.8579064165416</v>
       </c>
     </row>
@@ -2405,27 +2395,27 @@
         <v>79</v>
       </c>
       <c r="D53" s="8">
-        <f t="shared" ref="D53:I53" si="19">-(D5-C5)*$B$29</f>
+        <f t="shared" ref="D53:I53" si="22">-(D5-C5)*$B$29</f>
         <v>-41.55</v>
       </c>
       <c r="E53" s="8">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>-96.650832603490784</v>
       </c>
       <c r="F53" s="8">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>-110.13046239129453</v>
       </c>
       <c r="G53" s="8">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>-125.49005962812866</v>
       </c>
       <c r="H53" s="8">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>-142.99181828111614</v>
       </c>
       <c r="I53" s="8">
-        <f t="shared" si="19"/>
+        <f t="shared" si="22"/>
         <v>-162.93449979966863</v>
       </c>
     </row>
@@ -2434,27 +2424,27 @@
         <v>80</v>
       </c>
       <c r="D54" s="8">
-        <f t="shared" ref="D54:I54" si="20">-D5*$B$30*$B$31</f>
+        <f t="shared" ref="D54:I54" si="23">-D5*$B$30*$B$31</f>
         <v>0</v>
       </c>
       <c r="E54" s="8">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="F54" s="8">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="G54" s="8">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="H54" s="8">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
       <c r="I54" s="8">
-        <f t="shared" si="20"/>
+        <f t="shared" si="23"/>
         <v>0</v>
       </c>
     </row>
@@ -2463,27 +2453,27 @@
         <v>81</v>
       </c>
       <c r="D55" s="6">
-        <f t="shared" ref="D55:I55" si="21">D49+D50+D51+D52+D53+D54</f>
+        <f t="shared" ref="D55:I55" si="24">D49+D50+D51+D52+D53+D54</f>
         <v>807.22516216216206</v>
       </c>
       <c r="E55" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>961.9293085101375</v>
       </c>
       <c r="F55" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>1120.6594051989971</v>
       </c>
       <c r="G55" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>1322.350059421859</v>
       </c>
       <c r="H55" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>1573.4808698132258</v>
       </c>
       <c r="I55" s="6">
-        <f t="shared" si="21"/>
+        <f t="shared" si="24"/>
         <v>1761.5782403849648</v>
       </c>
     </row>
@@ -2550,27 +2540,27 @@
         <v>86</v>
       </c>
       <c r="D58" s="23">
-        <f t="shared" ref="D58:I58" si="22">1/(1+$B$23)^D57</f>
+        <f t="shared" ref="D58:I58" si="25">1/(1+$B$23)^D57</f>
         <v>0.99034982314742415</v>
       </c>
       <c r="E58" s="23">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0.93763146502673567</v>
       </c>
       <c r="F58" s="23">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0.85607156105907578</v>
       </c>
       <c r="G58" s="23">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0.78180051238271775</v>
       </c>
       <c r="H58" s="23">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0.71397307066914861</v>
       </c>
       <c r="I58" s="23">
-        <f t="shared" si="22"/>
+        <f t="shared" si="25"/>
         <v>0.65203020152433666</v>
       </c>
     </row>
@@ -2579,27 +2569,27 @@
         <v>87</v>
       </c>
       <c r="D59" s="6">
-        <f t="shared" ref="D59:I59" si="23">D55*D56*D58</f>
+        <f t="shared" ref="D59:I59" si="26">D55*D56*D58</f>
         <v>399.71764829372398</v>
       </c>
       <c r="E59" s="6">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>901.93518679051499</v>
       </c>
       <c r="F59" s="6">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>959.36464642424073</v>
       </c>
       <c r="G59" s="6">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1033.8139540053267</v>
       </c>
       <c r="H59" s="6">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1123.4229682597118</v>
       </c>
       <c r="I59" s="6">
-        <f t="shared" si="23"/>
+        <f t="shared" si="26"/>
         <v>1148.602215079095</v>
       </c>
     </row>
@@ -2608,27 +2598,27 @@
         <v>88</v>
       </c>
       <c r="D60" s="8">
-        <f t="shared" ref="D60:I60" si="24">-$B$37</f>
+        <f t="shared" ref="D60:I60" si="27">-$B$37</f>
         <v>-65</v>
       </c>
       <c r="E60" s="8">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>-65</v>
       </c>
       <c r="F60" s="8">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>-65</v>
       </c>
       <c r="G60" s="8">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>-65</v>
       </c>
       <c r="H60" s="8">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>-65</v>
       </c>
       <c r="I60" s="8">
-        <f t="shared" si="24"/>
+        <f t="shared" si="27"/>
         <v>-65</v>
       </c>
     </row>
@@ -2637,27 +2627,27 @@
         <v>89</v>
       </c>
       <c r="D61" s="8">
-        <f t="shared" ref="D61:I61" si="25">(D49+D60)*(1-$B$27)</f>
+        <f t="shared" ref="D61:I61" si="28">(D49+D60)*(1-$B$27)</f>
         <v>810.96016216216208</v>
       </c>
       <c r="E61" s="8">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>1027.9624966497215</v>
       </c>
       <c r="F61" s="8">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>1209.1075774234512</v>
       </c>
       <c r="G61" s="8">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>1437.1759732349046</v>
       </c>
       <c r="H61" s="8">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>1719.3166361631966</v>
       </c>
       <c r="I61" s="8">
-        <f t="shared" si="25"/>
+        <f t="shared" si="28"/>
         <v>1943.8349493954972</v>
       </c>
       <c r="J61" s="13" t="s">
@@ -2669,27 +2659,27 @@
         <v>91</v>
       </c>
       <c r="D62" s="24">
-        <f t="shared" ref="D62:I62" si="26">D61/$B$33</f>
+        <f t="shared" ref="D62:I62" si="29">D61/$B$33</f>
         <v>5.3003932167461576</v>
       </c>
       <c r="E62" s="24">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>6.7187091284295528</v>
       </c>
       <c r="F62" s="24">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>7.9026639047284393</v>
       </c>
       <c r="G62" s="24">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>9.3933070146072204</v>
       </c>
       <c r="H62" s="24">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>11.237363635053573</v>
       </c>
       <c r="I62" s="24">
-        <f t="shared" si="26"/>
+        <f t="shared" si="29"/>
         <v>12.704803590820243</v>
       </c>
       <c r="J62" s="13" t="s">
@@ -2935,26 +2925,26 @@
         <v>105</v>
       </c>
       <c r="B83" s="9"/>
-      <c r="C83" s="60">
+      <c r="C83" s="57">
         <f>C5</f>
         <v>4343</v>
       </c>
-      <c r="D83" s="57">
+      <c r="D83" s="54">
         <v>4625</v>
       </c>
-      <c r="E83" s="57">
+      <c r="E83" s="54">
         <v>4918</v>
       </c>
-      <c r="F83" s="57">
+      <c r="F83" s="54">
         <v>5263</v>
       </c>
-      <c r="G83" s="57">
+      <c r="G83" s="54">
         <v>5650</v>
       </c>
-      <c r="H83" s="57">
+      <c r="H83" s="54">
         <v>6088</v>
       </c>
-      <c r="I83" s="57">
+      <c r="I83" s="54">
         <v>6704</v>
       </c>
     </row>
@@ -2964,28 +2954,28 @@
       </c>
       <c r="B84" s="19"/>
       <c r="C84" s="19"/>
-      <c r="D84" s="58">
-        <f t="shared" ref="D84:I84" si="27">D83/C83-1</f>
+      <c r="D84" s="55">
+        <f t="shared" ref="D84:I84" si="30">D83/C83-1</f>
         <v>6.4932074602809031E-2</v>
       </c>
-      <c r="E84" s="58">
-        <f t="shared" si="27"/>
+      <c r="E84" s="55">
+        <f t="shared" si="30"/>
         <v>6.3351351351351282E-2</v>
       </c>
-      <c r="F84" s="58">
-        <f t="shared" si="27"/>
+      <c r="F84" s="55">
+        <f t="shared" si="30"/>
         <v>7.0150467669784389E-2</v>
       </c>
-      <c r="G84" s="58">
-        <f t="shared" si="27"/>
+      <c r="G84" s="55">
+        <f t="shared" si="30"/>
         <v>7.3532205966178932E-2</v>
       </c>
-      <c r="H84" s="58">
-        <f t="shared" si="27"/>
+      <c r="H84" s="55">
+        <f t="shared" si="30"/>
         <v>7.7522123893805306E-2</v>
       </c>
-      <c r="I84" s="58">
-        <f t="shared" si="27"/>
+      <c r="I84" s="55">
+        <f t="shared" si="30"/>
         <v>0.10118265440210239</v>
       </c>
     </row>
@@ -2995,22 +2985,22 @@
       </c>
       <c r="B85" s="19"/>
       <c r="C85" s="19"/>
-      <c r="D85" s="59">
+      <c r="D85" s="56">
         <v>0.68500000000000005</v>
       </c>
-      <c r="E85" s="59">
+      <c r="E85" s="56">
         <v>0.69099999999999995</v>
       </c>
-      <c r="F85" s="59">
+      <c r="F85" s="56">
         <v>0.69499999999999995</v>
       </c>
-      <c r="G85" s="59">
+      <c r="G85" s="56">
         <v>0.7</v>
       </c>
-      <c r="H85" s="59">
+      <c r="H85" s="56">
         <v>0.70299999999999996</v>
       </c>
-      <c r="I85" s="59">
+      <c r="I85" s="56">
         <v>0.70799999999999996</v>
       </c>
     </row>
@@ -3020,22 +3010,22 @@
       </c>
       <c r="B86" s="9"/>
       <c r="C86" s="9"/>
-      <c r="D86" s="57">
+      <c r="D86" s="54">
         <v>1299</v>
       </c>
-      <c r="E86" s="57">
+      <c r="E86" s="54">
         <v>1490</v>
       </c>
-      <c r="F86" s="57">
+      <c r="F86" s="54">
         <v>1623</v>
       </c>
-      <c r="G86" s="57">
+      <c r="G86" s="54">
         <v>1791</v>
       </c>
-      <c r="H86" s="57">
+      <c r="H86" s="54">
         <v>1997</v>
       </c>
-      <c r="I86" s="57">
+      <c r="I86" s="54">
         <v>2171</v>
       </c>
     </row>
@@ -3045,33 +3035,33 @@
       </c>
       <c r="B87" s="19"/>
       <c r="C87" s="19"/>
-      <c r="D87" s="58">
-        <f t="shared" ref="D87:I87" si="28">D86/D83</f>
+      <c r="D87" s="55">
+        <f t="shared" ref="D87:I87" si="31">D86/D83</f>
         <v>0.28086486486486484</v>
       </c>
-      <c r="E87" s="58">
-        <f t="shared" si="28"/>
+      <c r="E87" s="55">
+        <f t="shared" si="31"/>
         <v>0.3029686864579097</v>
       </c>
-      <c r="F87" s="58">
-        <f t="shared" si="28"/>
+      <c r="F87" s="55">
+        <f t="shared" si="31"/>
         <v>0.30837925137754135</v>
       </c>
-      <c r="G87" s="58">
-        <f t="shared" si="28"/>
+      <c r="G87" s="55">
+        <f t="shared" si="31"/>
         <v>0.31699115044247789</v>
       </c>
-      <c r="H87" s="58">
-        <f t="shared" si="28"/>
+      <c r="H87" s="55">
+        <f t="shared" si="31"/>
         <v>0.32802233902759526</v>
       </c>
-      <c r="I87" s="58">
-        <f t="shared" si="28"/>
+      <c r="I87" s="55">
+        <f t="shared" si="31"/>
         <v>0.32383651551312648</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A88" s="61" t="s">
+      <c r="A88" s="58" t="s">
         <v>104</v>
       </c>
     </row>

</xml_diff>